<commit_message>
Demonstração sem menções à área hospitalar
- setores e equipamentos de manutenção genéricos (Produção, Expedição, compressor, empilhadeira...)
- mesmo ajuste na API de teste, na planilha de teste e nos exemplos/comentários do assistente
- telas do portfólio refeitas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nomuo3bZrtv9jbtm4CbzHB
</commit_message>
<xml_diff>
--- a/exemplos/planilha-teste.xlsx
+++ b/exemplos/planilha-teste.xlsx
@@ -465,7 +465,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D6" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E6" t="str">
         <v>Calibração</v>
@@ -491,10 +491,10 @@
         <v>2026-07-23</v>
       </c>
       <c r="C7" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D7" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E7" t="str">
         <v>Calibração</v>
@@ -520,10 +520,10 @@
         <v>2026-07-22</v>
       </c>
       <c r="C8" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D8" t="str">
-        <v>Centro Cirúrgico</v>
+        <v>Expedição</v>
       </c>
       <c r="E8" t="str">
         <v>corretiva</v>
@@ -549,10 +549,10 @@
         <v>13/07/2026</v>
       </c>
       <c r="C9" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D9" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E9" t="str">
         <v>Corretiva</v>
@@ -578,10 +578,10 @@
         <v>15/07/2026</v>
       </c>
       <c r="C10" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D10" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E10" t="str">
         <v>corretiva</v>
@@ -607,10 +607,10 @@
         <v>26/7/26</v>
       </c>
       <c r="C11" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D11" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E11" t="str">
         <v>Calibração</v>
@@ -636,10 +636,10 @@
         <v>11/07/2026</v>
       </c>
       <c r="C12" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D12" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E12" t="str">
         <v>Calibração</v>
@@ -665,10 +665,10 @@
         <v>4/7/26</v>
       </c>
       <c r="C13" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D13" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E13" t="str">
         <v>Corretiva</v>
@@ -697,7 +697,7 @@
         <v>Gerador</v>
       </c>
       <c r="D14" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E14" t="str">
         <v>Calibração</v>
@@ -726,7 +726,7 @@
         <v>Gerador</v>
       </c>
       <c r="D15" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E15" t="str">
         <v>Preventiva</v>
@@ -752,10 +752,10 @@
         <v>2026-07-12</v>
       </c>
       <c r="C16" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D16" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E16" t="str">
         <v>Calibração</v>
@@ -781,10 +781,10 @@
         <v>3/7/26</v>
       </c>
       <c r="C17" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D17" t="str">
-        <v>Laboratório</v>
+        <v>Refeitório</v>
       </c>
       <c r="E17" t="str">
         <v>Preventiva</v>
@@ -810,10 +810,10 @@
         <v>2026-07-05</v>
       </c>
       <c r="C18" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D18" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E18" t="str">
         <v>corretiva</v>
@@ -839,10 +839,10 @@
         <v>2026-07-07</v>
       </c>
       <c r="C19" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D19" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E19" t="str">
         <v>Calibração</v>
@@ -868,10 +868,10 @@
         <v>15/7/26</v>
       </c>
       <c r="C20" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D20" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E20" t="str">
         <v>Corretiva</v>
@@ -897,10 +897,10 @@
         <v>02/07/2026</v>
       </c>
       <c r="C21" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D21" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E21" t="str">
         <v>Calibração</v>
@@ -926,10 +926,10 @@
         <v>19/7/26</v>
       </c>
       <c r="C22" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D22" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E22" t="str">
         <v>PREVENTIVA</v>
@@ -958,7 +958,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D23" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E23" t="str">
         <v>Preventiva</v>
@@ -984,10 +984,10 @@
         <v>2026-07-06</v>
       </c>
       <c r="C24" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D24" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E24" t="str">
         <v>Calibração</v>
@@ -1013,10 +1013,10 @@
         <v>15/7/26</v>
       </c>
       <c r="C25" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D25" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E25" t="str">
         <v>Calibração</v>
@@ -1042,10 +1042,10 @@
         <v>11/7/26</v>
       </c>
       <c r="C26" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D26" t="str">
-        <v>Centro Cirúrgico</v>
+        <v>Expedição</v>
       </c>
       <c r="E26" t="str">
         <v>corretiva</v>
@@ -1074,7 +1074,7 @@
         <v>Gerador</v>
       </c>
       <c r="D27" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E27" t="str">
         <v>Corretiva</v>
@@ -1103,7 +1103,7 @@
         <v>Gerador</v>
       </c>
       <c r="D28" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E28" t="str">
         <v>Preventiva</v>
@@ -1129,10 +1129,10 @@
         <v>2026-07-06</v>
       </c>
       <c r="C29" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D29" t="str">
-        <v>Centro Cirúrgico</v>
+        <v>Expedição</v>
       </c>
       <c r="E29" t="str">
         <v>PREVENTIVA</v>
@@ -1161,7 +1161,7 @@
         <v>Gerador</v>
       </c>
       <c r="D30" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E30" t="str">
         <v>corretiva</v>
@@ -1190,7 +1190,7 @@
         <v>Gerador</v>
       </c>
       <c r="D31" t="str">
-        <v>Laboratório</v>
+        <v>Refeitório</v>
       </c>
       <c r="E31" t="str">
         <v>Calibração</v>
@@ -1216,10 +1216,10 @@
         <v>20/7/26</v>
       </c>
       <c r="C32" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D32" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E32" t="str">
         <v>Corretiva</v>
@@ -1248,7 +1248,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D33" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E33" t="str">
         <v>PREVENTIVA</v>
@@ -1274,10 +1274,10 @@
         <v>26/07/2026</v>
       </c>
       <c r="C34" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D34" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E34" t="str">
         <v>Corretiva</v>
@@ -1303,10 +1303,10 @@
         <v>2/7/26</v>
       </c>
       <c r="C35" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D35" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E35" t="str">
         <v>Preventiva</v>
@@ -1332,10 +1332,10 @@
         <v>2026-07-14</v>
       </c>
       <c r="C36" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D36" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E36" t="str">
         <v>PREVENTIVA</v>
@@ -1361,10 +1361,10 @@
         <v>2026-07-14</v>
       </c>
       <c r="C37" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D37" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E37" t="str">
         <v>PREVENTIVA</v>
@@ -1390,10 +1390,10 @@
         <v>13/7/26</v>
       </c>
       <c r="C38" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D38" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E38" t="str">
         <v>Preventiva</v>
@@ -1419,10 +1419,10 @@
         <v>21/07/2026</v>
       </c>
       <c r="C39" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D39" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E39" t="str">
         <v>Calibração</v>
@@ -1451,7 +1451,7 @@
         <v>Gerador</v>
       </c>
       <c r="D40" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E40" t="str">
         <v>Calibração</v>
@@ -1480,7 +1480,7 @@
         <v>Gerador</v>
       </c>
       <c r="D41" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E41" t="str">
         <v>PREVENTIVA</v>
@@ -1506,10 +1506,10 @@
         <v>2026-07-21</v>
       </c>
       <c r="C42" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D42" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E42" t="str">
         <v>PREVENTIVA</v>
@@ -1535,10 +1535,10 @@
         <v>2026-07-26</v>
       </c>
       <c r="C43" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D43" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E43" t="str">
         <v>Corretiva</v>
@@ -1567,7 +1567,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D44" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E44" t="str">
         <v>Corretiva</v>
@@ -1596,7 +1596,7 @@
         <v>Gerador</v>
       </c>
       <c r="D45" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E45" t="str">
         <v>corretiva</v>
@@ -1622,10 +1622,10 @@
         <v>2026-07-07</v>
       </c>
       <c r="C46" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D46" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E46" t="str">
         <v>Corretiva</v>
@@ -1651,10 +1651,10 @@
         <v>15/08/2026</v>
       </c>
       <c r="C47" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D47" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E47" t="str">
         <v>Corretiva</v>
@@ -1680,10 +1680,10 @@
         <v>17/08/2026</v>
       </c>
       <c r="C48" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D48" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E48" t="str">
         <v>Preventiva</v>
@@ -1712,7 +1712,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D49" t="str">
-        <v>Centro Cirúrgico</v>
+        <v>Expedição</v>
       </c>
       <c r="E49" t="str">
         <v>corretiva</v>
@@ -1738,10 +1738,10 @@
         <v>23/08/2026</v>
       </c>
       <c r="C50" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D50" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E50" t="str">
         <v>Calibração</v>
@@ -1770,7 +1770,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D51" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E51" t="str">
         <v>Corretiva</v>
@@ -1796,10 +1796,10 @@
         <v>18/08/2026</v>
       </c>
       <c r="C52" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D52" t="str">
-        <v>Centro Cirúrgico</v>
+        <v>Expedição</v>
       </c>
       <c r="E52" t="str">
         <v>Calibração</v>
@@ -1828,7 +1828,7 @@
         <v>Gerador</v>
       </c>
       <c r="D53" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E53" t="str">
         <v>Corretiva</v>
@@ -1854,10 +1854,10 @@
         <v>2026-08-16</v>
       </c>
       <c r="C54" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D54" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E54" t="str">
         <v>Corretiva</v>
@@ -1883,10 +1883,10 @@
         <v>23/8/26</v>
       </c>
       <c r="C55" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D55" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E55" t="str">
         <v>Calibração</v>
@@ -1912,10 +1912,10 @@
         <v>23/08/2026</v>
       </c>
       <c r="C56" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D56" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E56" t="str">
         <v>Calibração</v>
@@ -1941,10 +1941,10 @@
         <v>11/8/26</v>
       </c>
       <c r="C57" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D57" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E57" t="str">
         <v>Calibração</v>
@@ -1973,7 +1973,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D58" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E58" t="str">
         <v>PREVENTIVA</v>
@@ -2002,7 +2002,7 @@
         <v>Gerador</v>
       </c>
       <c r="D59" t="str">
-        <v>Laboratório</v>
+        <v>Refeitório</v>
       </c>
       <c r="E59" t="str">
         <v>Calibração</v>
@@ -2031,7 +2031,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D60" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E60" t="str">
         <v>PREVENTIVA</v>
@@ -2057,10 +2057,10 @@
         <v>20/08/2026</v>
       </c>
       <c r="C61" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D61" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E61" t="str">
         <v>Preventiva</v>
@@ -2089,7 +2089,7 @@
         <v>Gerador</v>
       </c>
       <c r="D62" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E62" t="str">
         <v>PREVENTIVA</v>
@@ -2115,10 +2115,10 @@
         <v>15/08/2026</v>
       </c>
       <c r="C63" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D63" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E63" t="str">
         <v>PREVENTIVA</v>
@@ -2144,10 +2144,10 @@
         <v>2026-08-11</v>
       </c>
       <c r="C64" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D64" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E64" t="str">
         <v>corretiva</v>
@@ -2173,10 +2173,10 @@
         <v>2026-08-04</v>
       </c>
       <c r="C65" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D65" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E65" t="str">
         <v>Calibração</v>
@@ -2202,10 +2202,10 @@
         <v>2/8/26</v>
       </c>
       <c r="C66" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D66" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E66" t="str">
         <v>corretiva</v>
@@ -2231,10 +2231,10 @@
         <v>14/08/2026</v>
       </c>
       <c r="C68" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D68" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E68" t="str">
         <v>PREVENTIVA</v>
@@ -2260,10 +2260,10 @@
         <v>12/08/2026</v>
       </c>
       <c r="C69" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D69" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E69" t="str">
         <v>Corretiva</v>
@@ -2292,7 +2292,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D70" t="str">
-        <v>Centro Cirúrgico</v>
+        <v>Expedição</v>
       </c>
       <c r="E70" t="str">
         <v>PREVENTIVA</v>
@@ -2321,7 +2321,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D71" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E71" t="str">
         <v>PREVENTIVA</v>
@@ -2350,7 +2350,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D72" t="str">
-        <v>Laboratório</v>
+        <v>Refeitório</v>
       </c>
       <c r="E72" t="str">
         <v>Preventiva</v>
@@ -2379,7 +2379,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D73" t="str">
-        <v>Centro Cirúrgico</v>
+        <v>Expedição</v>
       </c>
       <c r="E73" t="str">
         <v>corretiva</v>
@@ -2408,7 +2408,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D74" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E74" t="str">
         <v>Corretiva</v>
@@ -2434,10 +2434,10 @@
         <v>2026-08-02</v>
       </c>
       <c r="C75" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D75" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E75" t="str">
         <v>Corretiva</v>
@@ -2463,10 +2463,10 @@
         <v>15/8/26</v>
       </c>
       <c r="C76" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D76" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E76" t="str">
         <v>Corretiva</v>
@@ -2492,10 +2492,10 @@
         <v>2026-08-23</v>
       </c>
       <c r="C77" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D77" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E77" t="str">
         <v>corretiva</v>
@@ -2521,10 +2521,10 @@
         <v>2026-08-19</v>
       </c>
       <c r="C78" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D78" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E78" t="str">
         <v>Calibração</v>
@@ -2553,7 +2553,7 @@
         <v>Gerador</v>
       </c>
       <c r="D79" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E79" t="str">
         <v>Calibração</v>
@@ -2579,10 +2579,10 @@
         <v>01/08/2026</v>
       </c>
       <c r="C80" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D80" t="str">
-        <v>Centro Cirúrgico</v>
+        <v>Expedição</v>
       </c>
       <c r="E80" t="str">
         <v>Preventiva</v>
@@ -2608,10 +2608,10 @@
         <v>2026-08-18</v>
       </c>
       <c r="C81" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D81" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E81" t="str">
         <v>Preventiva</v>
@@ -2640,7 +2640,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D82" t="str">
-        <v>Laboratório</v>
+        <v>Refeitório</v>
       </c>
       <c r="E82" t="str">
         <v>Calibração</v>
@@ -2666,10 +2666,10 @@
         <v>17/8/26</v>
       </c>
       <c r="C83" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D83" t="str">
-        <v>Laboratório</v>
+        <v>Refeitório</v>
       </c>
       <c r="E83" t="str">
         <v>PREVENTIVA</v>
@@ -2695,10 +2695,10 @@
         <v>8/8/26</v>
       </c>
       <c r="C84" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D84" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E84" t="str">
         <v>Corretiva</v>
@@ -2724,10 +2724,10 @@
         <v>16/08/2026</v>
       </c>
       <c r="C85" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D85" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E85" t="str">
         <v>corretiva</v>
@@ -2753,10 +2753,10 @@
         <v>16/08/2026</v>
       </c>
       <c r="C86" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D86" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E86" t="str">
         <v>corretiva</v>
@@ -2782,10 +2782,10 @@
         <v>2026-08-04</v>
       </c>
       <c r="C87" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D87" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E87" t="str">
         <v>Corretiva</v>
@@ -2811,10 +2811,10 @@
         <v>01/08/2026</v>
       </c>
       <c r="C88" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D88" t="str">
-        <v>Laboratório</v>
+        <v>Refeitório</v>
       </c>
       <c r="E88" t="str">
         <v>PREVENTIVA</v>
@@ -2843,7 +2843,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D89" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E89" t="str">
         <v>PREVENTIVA</v>
@@ -2872,7 +2872,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D90" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E90" t="str">
         <v>Preventiva</v>
@@ -2898,10 +2898,10 @@
         <v>11/09/2026</v>
       </c>
       <c r="C91" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D91" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E91" t="str">
         <v>PREVENTIVA</v>
@@ -2927,10 +2927,10 @@
         <v>14/09/2026</v>
       </c>
       <c r="C92" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D92" t="str">
-        <v>Centro Cirúrgico</v>
+        <v>Expedição</v>
       </c>
       <c r="E92" t="str">
         <v>Calibração</v>
@@ -2956,10 +2956,10 @@
         <v>2026-09-14</v>
       </c>
       <c r="C93" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D93" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E93" t="str">
         <v>Preventiva</v>
@@ -2985,10 +2985,10 @@
         <v>24/9/26</v>
       </c>
       <c r="C94" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D94" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E94" t="str">
         <v>Corretiva</v>
@@ -3014,10 +3014,10 @@
         <v>17/09/2026</v>
       </c>
       <c r="C95" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D95" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E95" t="str">
         <v>Calibração</v>
@@ -3043,10 +3043,10 @@
         <v>2026-09-02</v>
       </c>
       <c r="C96" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D96" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E96" t="str">
         <v>Corretiva</v>
@@ -3072,10 +3072,10 @@
         <v>15/09/2026</v>
       </c>
       <c r="C97" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D97" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E97" t="str">
         <v>corretiva</v>
@@ -3101,10 +3101,10 @@
         <v>19/9/26</v>
       </c>
       <c r="C98" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D98" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E98" t="str">
         <v>corretiva</v>
@@ -3130,10 +3130,10 @@
         <v>10/09/2026</v>
       </c>
       <c r="C99" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D99" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E99" t="str">
         <v>Preventiva</v>
@@ -3159,10 +3159,10 @@
         <v>2026-09-25</v>
       </c>
       <c r="C100" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D100" t="str">
-        <v>Laboratório</v>
+        <v>Refeitório</v>
       </c>
       <c r="E100" t="str">
         <v>corretiva</v>
@@ -3191,7 +3191,7 @@
         <v>Gerador</v>
       </c>
       <c r="D101" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E101" t="str">
         <v>Calibração</v>
@@ -3217,10 +3217,10 @@
         <v>6/9/26</v>
       </c>
       <c r="C102" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D102" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E102" t="str">
         <v>Calibração</v>
@@ -3246,10 +3246,10 @@
         <v>13/9/26</v>
       </c>
       <c r="C103" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D103" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E103" t="str">
         <v>corretiva</v>
@@ -3278,7 +3278,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D104" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E104" t="str">
         <v>PREVENTIVA</v>
@@ -3307,7 +3307,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D105" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E105" t="str">
         <v>corretiva</v>
@@ -3333,10 +3333,10 @@
         <v>2026-09-26</v>
       </c>
       <c r="C106" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D106" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E106" t="str">
         <v>Corretiva</v>
@@ -3362,10 +3362,10 @@
         <v>07/09/2026</v>
       </c>
       <c r="C107" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D107" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E107" t="str">
         <v>Calibração</v>
@@ -3391,10 +3391,10 @@
         <v>20/9/26</v>
       </c>
       <c r="C108" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D108" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E108" t="str">
         <v>Calibração</v>
@@ -3420,10 +3420,10 @@
         <v>9/9/26</v>
       </c>
       <c r="C109" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D109" t="str">
-        <v>Centro Cirúrgico</v>
+        <v>Expedição</v>
       </c>
       <c r="E109" t="str">
         <v>PREVENTIVA</v>
@@ -3449,10 +3449,10 @@
         <v>6/9/26</v>
       </c>
       <c r="C110" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D110" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E110" t="str">
         <v>corretiva</v>
@@ -3478,10 +3478,10 @@
         <v>19/09/2026</v>
       </c>
       <c r="C111" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D111" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E111" t="str">
         <v>PREVENTIVA</v>
@@ -3510,7 +3510,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D112" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E112" t="str">
         <v>PREVENTIVA</v>
@@ -3536,10 +3536,10 @@
         <v>03/09/2026</v>
       </c>
       <c r="C113" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D113" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E113" t="str">
         <v>Calibração</v>
@@ -3565,10 +3565,10 @@
         <v>27/09/2026</v>
       </c>
       <c r="C114" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D114" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E114" t="str">
         <v>Corretiva</v>
@@ -3594,10 +3594,10 @@
         <v>21/9/26</v>
       </c>
       <c r="C115" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D115" t="str">
-        <v>Laboratório</v>
+        <v>Refeitório</v>
       </c>
       <c r="E115" t="str">
         <v>Corretiva</v>
@@ -3623,10 +3623,10 @@
         <v>02/09/2026</v>
       </c>
       <c r="C116" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D116" t="str">
-        <v>Centro Cirúrgico</v>
+        <v>Expedição</v>
       </c>
       <c r="E116" t="str">
         <v>PREVENTIVA</v>
@@ -3652,10 +3652,10 @@
         <v>7/9/26</v>
       </c>
       <c r="C117" t="str">
-        <v>Desfibrilador</v>
+        <v>Esteira transportadora</v>
       </c>
       <c r="D117" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E117" t="str">
         <v>PREVENTIVA</v>
@@ -3684,7 +3684,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D118" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E118" t="str">
         <v>corretiva</v>
@@ -3710,10 +3710,10 @@
         <v>13/9/26</v>
       </c>
       <c r="C119" t="str">
-        <v>Bomba de infusão</v>
+        <v>Bomba d'água</v>
       </c>
       <c r="D119" t="str">
-        <v>laboratorio</v>
+        <v>refeitorio</v>
       </c>
       <c r="E119" t="str">
         <v>PREVENTIVA</v>
@@ -3742,7 +3742,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D120" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E120" t="str">
         <v>Calibração</v>
@@ -3768,10 +3768,10 @@
         <v>26/9/26</v>
       </c>
       <c r="C121" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D121" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E121" t="str">
         <v>corretiva</v>
@@ -3797,10 +3797,10 @@
         <v>7/9/26</v>
       </c>
       <c r="C122" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D122" t="str">
-        <v>Pronto Atendimento</v>
+        <v>Almoxarifado</v>
       </c>
       <c r="E122" t="str">
         <v>Calibração</v>
@@ -3826,10 +3826,10 @@
         <v>2026-09-28</v>
       </c>
       <c r="C123" t="str">
-        <v>Monitor multiparâmetro</v>
+        <v>Compressor de ar</v>
       </c>
       <c r="D123" t="str">
-        <v>UTI Adulto</v>
+        <v>Produção</v>
       </c>
       <c r="E123" t="str">
         <v>Corretiva</v>
@@ -3858,7 +3858,7 @@
         <v>Gerador</v>
       </c>
       <c r="D124" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E124" t="str">
         <v>Corretiva</v>
@@ -3884,10 +3884,10 @@
         <v>19/9/26</v>
       </c>
       <c r="C125" t="str">
-        <v>Ventilador pulmonar</v>
+        <v>Empilhadeira</v>
       </c>
       <c r="D125" t="str">
-        <v>CENTRO CIRURGICO</v>
+        <v>EXPEDICAO</v>
       </c>
       <c r="E125" t="str">
         <v>Corretiva</v>
@@ -3916,7 +3916,7 @@
         <v>Gerador</v>
       </c>
       <c r="D126" t="str">
-        <v>Radiologia</v>
+        <v>Administrativo</v>
       </c>
       <c r="E126" t="str">
         <v>PREVENTIVA</v>
@@ -3942,10 +3942,10 @@
         <v>2026-09-22</v>
       </c>
       <c r="C127" t="str">
-        <v>Autoclave</v>
+        <v>Caldeira</v>
       </c>
       <c r="D127" t="str">
-        <v>uti adulto</v>
+        <v>produção</v>
       </c>
       <c r="E127" t="str">
         <v>corretiva</v>
@@ -3974,7 +3974,7 @@
         <v>Ar-condicionado</v>
       </c>
       <c r="D128" t="str">
-        <v>Laboratório</v>
+        <v>Refeitório</v>
       </c>
       <c r="E128" t="str">
         <v>Corretiva</v>

</xml_diff>